<commit_message>
Added the BMW page
</commit_message>
<xml_diff>
--- a/Excel/testdata.xlsx
+++ b/Excel/testdata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\PythonProgramming\PageObjectModelFramework\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{365DEAA4-6F4A-455F-9D23-0198789B589A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70FF2AFD-041D-4EE5-AA7E-267F8E7B495A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{9E2CB3D1-0571-491D-BF66-F783525DBCC6}"/>
+    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{9E2CB3D1-0571-491D-BF66-F783525DBCC6}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginTest" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>name</t>
   </si>
@@ -95,6 +95,12 @@
   </si>
   <si>
     <t>Maruti Cars</t>
+  </si>
+  <si>
+    <t>BMW</t>
+  </si>
+  <si>
+    <t>BMW Cars</t>
   </si>
 </sst>
 </file>
@@ -516,7 +522,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C31209CD-93B8-4CBE-97B4-1AD94EFBB0DE}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.21875" bestFit="1" customWidth="1"/>
@@ -563,6 +569,14 @@
         <v>22</v>
       </c>
     </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>